<commit_message>
Actualización de documentos + Arreglo de título
</commit_message>
<xml_diff>
--- a/FASE 2/EVIDENCIAS PROYECTO/EVIDENCIAS DE DOCUMENTACION/7- Pruebas y evidencias/Registro_Ejecucion_Pruebas_CultureGo.xlsx
+++ b/FASE 2/EVIDENCIAS PROYECTO/EVIDENCIAS DE DOCUMENTACION/7- Pruebas y evidencias/Registro_Ejecucion_Pruebas_CultureGo.xlsx
@@ -9437,10 +9437,10 @@
         <v>368</v>
       </c>
       <c r="D6" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="F6" s="24" t="n">
         <v>0.237</v>

</xml_diff>